<commit_message>
feat: add elemental tuning cards
</commit_message>
<xml_diff>
--- a/config/FantasyCard_Config.xlsx
+++ b/config/FantasyCard_Config.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_README" sheetId="1" r:id="R03a83947ce604924"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="2" r:id="R58033d761d1449a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CardLevels" sheetId="3" r:id="R74a7bc0e7457466d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monsters" sheetId="4" r:id="R105510f812d94757"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterIntents" sheetId="5" r:id="R34710e323d574fc7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EquipmentQuality" sheetId="6" r:id="R5c7481bd93b144cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backpacks" sheetId="7" r:id="R07966bfcb2cc4a2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LootRules" sheetId="8" r:id="Rf70f886f05054341"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Economy" sheetId="9" r:id="R7917a8ebbad34435"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MapTemplates" sheetId="10" r:id="Rbc37208eba9a4c4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BotTuning" sheetId="11" r:id="R0a2cd6bc7e9e44c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ShopCardPrices" sheetId="12" r:id="R2ba9d7d9485d40ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="13" r:id="Rc2b165d122af4491"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_README" sheetId="1" r:id="R18397e4dd2f54571"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="2" r:id="R4f4c0111e8c44e5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CardLevels" sheetId="3" r:id="R7edb50c473384c33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monsters" sheetId="4" r:id="Rcf6deb726ad2481f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterIntents" sheetId="5" r:id="R584031ff52c04ae3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EquipmentQuality" sheetId="6" r:id="R78006436d2a34199"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backpacks" sheetId="7" r:id="Rf35b73f25b5f4d29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LootRules" sheetId="8" r:id="R4e3b41b479424ad4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Economy" sheetId="9" r:id="R0b8ad12cc1e3478c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MapTemplates" sheetId="10" r:id="R52b408d97601403e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BotTuning" sheetId="11" r:id="R47647994d02d4d50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ShopCardPrices" sheetId="12" r:id="Rc4e1fa70431a47dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="13" r:id="R1476ea8a2f244eb5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1351,8 +1351,7 @@
         <x:v>卡牌基础定义；效果脚本 ID 仍由程序实现</x:v>
       </x:c>
       <x:c r="C5" s="24" t="n">
-        <x:f>COUNTA('Cards'!A6:A205)</x:f>
-        <x:v>200</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="E5" s="38" t="str">
         <x:v>权威状态机</x:v>
@@ -1369,8 +1368,7 @@
         <x:v>卡牌等级成长；一行对应一张卡的一个等级</x:v>
       </x:c>
       <x:c r="C6" s="27" t="n">
-        <x:f>COUNTA('CardLevels'!A6:A205)</x:f>
-        <x:v>200</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="E6" s="40" t="str">
         <x:v>战斗公式流程</x:v>
@@ -2180,7 +2178,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3408f2742935446f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10e517a74f4d4795"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2613,7 +2611,7 @@
         <x:v>Initial / Class / General / Monster</x:v>
       </x:c>
       <x:c r="D5" s="107" t="str">
-        <x:v>Damage / Heal / Assist</x:v>
+        <x:v>Damage / Heal / Assist / ElementTune</x:v>
       </x:c>
       <x:c r="E5" s="107" t="str">
         <x:v>职业卡限定职业</x:v>
@@ -21404,6 +21402,1786 @@
       <x:c r="AE217" s="77" t="str">
         <x:v>Metal</x:v>
       </x:c>
+    </x:row>
+    <x:row r="218">
+      <x:c r="A218" t="str">
+        <x:v>ET-FIRE-W</x:v>
+      </x:c>
+      <x:c r="B218" t="str">
+        <x:v>调焰</x:v>
+      </x:c>
+      <x:c r="C218" t="str">
+        <x:v>General</x:v>
+      </x:c>
+      <x:c r="D218" t="str">
+        <x:v>ElementTune</x:v>
+      </x:c>
+      <x:c r="E218"/>
+      <x:c r="F218"/>
+      <x:c r="G218" t="str">
+        <x:v>White</x:v>
+      </x:c>
+      <x:c r="H218" t="str">
+        <x:v>Fire</x:v>
+      </x:c>
+      <x:c r="I218" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J218" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K218" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L218" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M218" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N218" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O218" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P218" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q218" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R218" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S218" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T218" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U218" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="V218" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W218" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X218" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y218" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Z218" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AA218" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="AB218" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="AC218" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AD218" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AE218"/>
+    </x:row>
+    <x:row r="219">
+      <x:c r="A219" t="str">
+        <x:v>ET-FIRE-G</x:v>
+      </x:c>
+      <x:c r="B219" t="str">
+        <x:v>引焰</x:v>
+      </x:c>
+      <x:c r="C219" t="str">
+        <x:v>General</x:v>
+      </x:c>
+      <x:c r="D219" t="str">
+        <x:v>ElementTune</x:v>
+      </x:c>
+      <x:c r="E219"/>
+      <x:c r="F219"/>
+      <x:c r="G219" t="str">
+        <x:v>Green</x:v>
+      </x:c>
+      <x:c r="H219" t="str">
+        <x:v>Fire</x:v>
+      </x:c>
+      <x:c r="I219" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J219" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K219" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L219" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M219" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N219" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O219" t="n">
+        <x:v>-0.15</x:v>
+      </x:c>
+      <x:c r="P219" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="Q219" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R219" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S219" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T219" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U219" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="V219" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W219" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X219" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y219" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Z219" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AA219" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="AB219" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="AC219" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AD219" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AE219"/>
+    </x:row>
+    <x:row r="220">
+      <x:c r="A220" t="str">
+        <x:v>ET-FIRE-B</x:v>
+      </x:c>
+      <x:c r="B220" t="str">
+        <x:v>炽律</x:v>
+      </x:c>
+      <x:c r="C220" t="str">
+        <x:v>General</x:v>
+      </x:c>
+      <x:c r="D220" t="str">
+        <x:v>ElementTune</x:v>
+      </x:c>
+      <x:c r="E220"/>
+      <x:c r="F220"/>
+      <x:c r="G220" t="str">
+        <x:v>Blue</x:v>
+      </x:c>
+      <x:c r="H220" t="str">
+        <x:v>Fire</x:v>
+      </x:c>
+      <x:c r="I220" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="J220" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K220" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L220" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M220" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N220" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O220" t="n">
+        <x:v>-0.25</x:v>
+      </x:c>
+      <x:c r="P220" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="Q220" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R220" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S220" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T220" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U220" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="V220" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W220" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X220" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y220" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Z220" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AA220" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AB220" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AC220" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AD220" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AE220"/>
+    </x:row>
+    <x:row r="221">
+      <x:c r="A221" t="str">
+        <x:v>ET-FIRE-P</x:v>
+      </x:c>
+      <x:c r="B221" t="str">
+        <x:v>炎脉合奏</x:v>
+      </x:c>
+      <x:c r="C221" t="str">
+        <x:v>General</x:v>
+      </x:c>
+      <x:c r="D221" t="str">
+        <x:v>ElementTune</x:v>
+      </x:c>
+      <x:c r="E221"/>
+      <x:c r="F221"/>
+      <x:c r="G221" t="str">
+        <x:v>Purple</x:v>
+      </x:c>
+      <x:c r="H221" t="str">
+        <x:v>Fire</x:v>
+      </x:c>
+      <x:c r="I221" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="J221" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K221" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L221" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M221" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N221" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O221" t="n">
+        <x:v>-0.35</x:v>
+      </x:c>
+      <x:c r="P221" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="Q221" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R221" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S221" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T221" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U221" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="V221" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W221" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X221" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y221" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Z221" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AA221" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="AB221" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="AC221" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AD221" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AE221"/>
+    </x:row>
+    <x:row r="222">
+      <x:c r="A222" t="str">
+        <x:v>ET-WOOD-W</x:v>
+      </x:c>
+      <x:c r="B222" t="str">
+        <x:v>理枝</x:v>
+      </x:c>
+      <x:c r="C222" t="str">
+        <x:v>General</x:v>
+      </x:c>
+      <x:c r="D222" t="str">
+        <x:v>ElementTune</x:v>
+      </x:c>
+      <x:c r="E222"/>
+      <x:c r="F222"/>
+      <x:c r="G222" t="str">
+        <x:v>White</x:v>
+      </x:c>
+      <x:c r="H222" t="str">
+        <x:v>Wood</x:v>
+      </x:c>
+      <x:c r="I222" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J222" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K222" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L222" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M222" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N222" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O222" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P222" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q222" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R222" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S222" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T222" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U222" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="V222" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W222" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X222" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y222" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Z222" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AA222" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="AB222" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="AC222" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AD222" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AE222"/>
+    </x:row>
+    <x:row r="223">
+      <x:c r="A223" t="str">
+        <x:v>ET-WOOD-G</x:v>
+      </x:c>
+      <x:c r="B223" t="str">
+        <x:v>引芽</x:v>
+      </x:c>
+      <x:c r="C223" t="str">
+        <x:v>General</x:v>
+      </x:c>
+      <x:c r="D223" t="str">
+        <x:v>ElementTune</x:v>
+      </x:c>
+      <x:c r="E223"/>
+      <x:c r="F223"/>
+      <x:c r="G223" t="str">
+        <x:v>Green</x:v>
+      </x:c>
+      <x:c r="H223" t="str">
+        <x:v>Wood</x:v>
+      </x:c>
+      <x:c r="I223" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J223" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K223" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L223" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M223" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="N223" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O223" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P223" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q223" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R223" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S223" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T223" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U223" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="V223" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W223" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X223" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y223" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Z223" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AA223" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="AB223" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="AC223" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AD223" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AE223"/>
+    </x:row>
+    <x:row r="224">
+      <x:c r="A224" t="str">
+        <x:v>ET-WOOD-B</x:v>
+      </x:c>
+      <x:c r="B224" t="str">
+        <x:v>森息</x:v>
+      </x:c>
+      <x:c r="C224" t="str">
+        <x:v>General</x:v>
+      </x:c>
+      <x:c r="D224" t="str">
+        <x:v>ElementTune</x:v>
+      </x:c>
+      <x:c r="E224"/>
+      <x:c r="F224"/>
+      <x:c r="G224" t="str">
+        <x:v>Blue</x:v>
+      </x:c>
+      <x:c r="H224" t="str">
+        <x:v>Wood</x:v>
+      </x:c>
+      <x:c r="I224" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="J224" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K224" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L224" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M224" t="n">
+        <x:v>0.7</x:v>
+      </x:c>
+      <x:c r="N224" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O224" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P224" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q224" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R224" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S224" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T224" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U224" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="V224" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W224" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X224" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y224" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Z224" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AA224" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AB224" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AC224" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AD224" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AE224"/>
+    </x:row>
+    <x:row r="225">
+      <x:c r="A225" t="str">
+        <x:v>ET-WOOD-P</x:v>
+      </x:c>
+      <x:c r="B225" t="str">
+        <x:v>万木同频</x:v>
+      </x:c>
+      <x:c r="C225" t="str">
+        <x:v>General</x:v>
+      </x:c>
+      <x:c r="D225" t="str">
+        <x:v>ElementTune</x:v>
+      </x:c>
+      <x:c r="E225"/>
+      <x:c r="F225"/>
+      <x:c r="G225" t="str">
+        <x:v>Purple</x:v>
+      </x:c>
+      <x:c r="H225" t="str">
+        <x:v>Wood</x:v>
+      </x:c>
+      <x:c r="I225" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="J225" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K225" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L225" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M225" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N225" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O225" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P225" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q225" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R225" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S225" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T225" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U225" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="V225" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W225" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X225" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y225" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Z225" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AA225" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="AB225" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="AC225" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AD225" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AE225"/>
+    </x:row>
+    <x:row r="226">
+      <x:c r="A226" t="str">
+        <x:v>ET-EARTH-W</x:v>
+      </x:c>
+      <x:c r="B226" t="str">
+        <x:v>定土</x:v>
+      </x:c>
+      <x:c r="C226" t="str">
+        <x:v>General</x:v>
+      </x:c>
+      <x:c r="D226" t="str">
+        <x:v>ElementTune</x:v>
+      </x:c>
+      <x:c r="E226"/>
+      <x:c r="F226"/>
+      <x:c r="G226" t="str">
+        <x:v>White</x:v>
+      </x:c>
+      <x:c r="H226" t="str">
+        <x:v>Earth</x:v>
+      </x:c>
+      <x:c r="I226" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J226" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K226" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L226" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M226" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N226" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O226" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P226" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q226" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R226" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S226" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T226" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U226" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="V226" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W226" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X226" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y226" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Z226" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AA226" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="AB226" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="AC226" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AD226" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AE226"/>
+    </x:row>
+    <x:row r="227">
+      <x:c r="A227" t="str">
+        <x:v>ET-EARTH-G</x:v>
+      </x:c>
+      <x:c r="B227" t="str">
+        <x:v>护脉</x:v>
+      </x:c>
+      <x:c r="C227" t="str">
+        <x:v>General</x:v>
+      </x:c>
+      <x:c r="D227" t="str">
+        <x:v>ElementTune</x:v>
+      </x:c>
+      <x:c r="E227"/>
+      <x:c r="F227"/>
+      <x:c r="G227" t="str">
+        <x:v>Green</x:v>
+      </x:c>
+      <x:c r="H227" t="str">
+        <x:v>Earth</x:v>
+      </x:c>
+      <x:c r="I227" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J227" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K227" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L227" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="M227" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N227" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O227" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P227" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q227" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R227" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S227" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T227" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U227" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="V227" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W227" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X227" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y227" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Z227" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AA227" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="AB227" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="AC227" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AD227" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AE227"/>
+    </x:row>
+    <x:row r="228">
+      <x:c r="A228" t="str">
+        <x:v>ET-EARTH-B</x:v>
+      </x:c>
+      <x:c r="B228" t="str">
+        <x:v>地垒</x:v>
+      </x:c>
+      <x:c r="C228" t="str">
+        <x:v>General</x:v>
+      </x:c>
+      <x:c r="D228" t="str">
+        <x:v>ElementTune</x:v>
+      </x:c>
+      <x:c r="E228"/>
+      <x:c r="F228"/>
+      <x:c r="G228" t="str">
+        <x:v>Blue</x:v>
+      </x:c>
+      <x:c r="H228" t="str">
+        <x:v>Earth</x:v>
+      </x:c>
+      <x:c r="I228" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="J228" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K228" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L228" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="M228" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N228" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O228" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P228" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q228" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R228" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S228" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T228" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U228" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="V228" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W228" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X228" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y228" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Z228" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AA228" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AB228" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AC228" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AD228" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AE228"/>
+    </x:row>
+    <x:row r="229">
+      <x:c r="A229" t="str">
+        <x:v>ET-EARTH-P</x:v>
+      </x:c>
+      <x:c r="B229" t="str">
+        <x:v>山岳同调</x:v>
+      </x:c>
+      <x:c r="C229" t="str">
+        <x:v>General</x:v>
+      </x:c>
+      <x:c r="D229" t="str">
+        <x:v>ElementTune</x:v>
+      </x:c>
+      <x:c r="E229"/>
+      <x:c r="F229"/>
+      <x:c r="G229" t="str">
+        <x:v>Purple</x:v>
+      </x:c>
+      <x:c r="H229" t="str">
+        <x:v>Earth</x:v>
+      </x:c>
+      <x:c r="I229" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="J229" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K229" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L229" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="M229" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N229" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O229" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P229" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q229" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R229" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S229" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T229" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U229" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="V229" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W229" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X229" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y229" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Z229" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AA229" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="AB229" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="AC229" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AD229" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AE229"/>
+    </x:row>
+    <x:row r="230">
+      <x:c r="A230" t="str">
+        <x:v>ET-METAL-W</x:v>
+      </x:c>
+      <x:c r="B230" t="str">
+        <x:v>鸣金</x:v>
+      </x:c>
+      <x:c r="C230" t="str">
+        <x:v>General</x:v>
+      </x:c>
+      <x:c r="D230" t="str">
+        <x:v>ElementTune</x:v>
+      </x:c>
+      <x:c r="E230"/>
+      <x:c r="F230"/>
+      <x:c r="G230" t="str">
+        <x:v>White</x:v>
+      </x:c>
+      <x:c r="H230" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="I230" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J230" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K230" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L230" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M230" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N230" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O230" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P230" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q230" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R230" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S230" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T230" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U230" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="V230" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W230" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X230" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y230" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Z230" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AA230" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="AB230" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="AC230" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AD230" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AE230"/>
+    </x:row>
+    <x:row r="231">
+      <x:c r="A231" t="str">
+        <x:v>ET-METAL-G</x:v>
+      </x:c>
+      <x:c r="B231" t="str">
+        <x:v>锐音</x:v>
+      </x:c>
+      <x:c r="C231" t="str">
+        <x:v>General</x:v>
+      </x:c>
+      <x:c r="D231" t="str">
+        <x:v>ElementTune</x:v>
+      </x:c>
+      <x:c r="E231"/>
+      <x:c r="F231"/>
+      <x:c r="G231" t="str">
+        <x:v>Green</x:v>
+      </x:c>
+      <x:c r="H231" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="I231" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J231" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K231" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L231" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M231" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N231" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O231" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P231" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q231" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="R231" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S231" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T231" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U231" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="V231" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W231" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X231" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y231" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Z231" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AA231" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="AB231" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="AC231" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AD231" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AE231"/>
+    </x:row>
+    <x:row r="232">
+      <x:c r="A232" t="str">
+        <x:v>ET-METAL-B</x:v>
+      </x:c>
+      <x:c r="B232" t="str">
+        <x:v>金律</x:v>
+      </x:c>
+      <x:c r="C232" t="str">
+        <x:v>General</x:v>
+      </x:c>
+      <x:c r="D232" t="str">
+        <x:v>ElementTune</x:v>
+      </x:c>
+      <x:c r="E232"/>
+      <x:c r="F232"/>
+      <x:c r="G232" t="str">
+        <x:v>Blue</x:v>
+      </x:c>
+      <x:c r="H232" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="I232" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="J232" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K232" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L232" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M232" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N232" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O232" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P232" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q232" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R232" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S232" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T232" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U232" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="V232" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W232" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X232" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y232" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Z232" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AA232" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AB232" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AC232" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AD232" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AE232"/>
+    </x:row>
+    <x:row r="233">
+      <x:c r="A233" t="str">
+        <x:v>ET-METAL-P</x:v>
+      </x:c>
+      <x:c r="B233" t="str">
+        <x:v>天钟共鸣</x:v>
+      </x:c>
+      <x:c r="C233" t="str">
+        <x:v>General</x:v>
+      </x:c>
+      <x:c r="D233" t="str">
+        <x:v>ElementTune</x:v>
+      </x:c>
+      <x:c r="E233"/>
+      <x:c r="F233"/>
+      <x:c r="G233" t="str">
+        <x:v>Purple</x:v>
+      </x:c>
+      <x:c r="H233" t="str">
+        <x:v>Metal</x:v>
+      </x:c>
+      <x:c r="I233" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="J233" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K233" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L233" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M233" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N233" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O233" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P233" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q233" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="R233" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S233" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T233" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U233" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="V233" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W233" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X233" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y233" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Z233" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AA233" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="AB233" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="AC233" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AD233" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AE233"/>
+    </x:row>
+    <x:row r="234">
+      <x:c r="A234" t="str">
+        <x:v>ET-WATER-W</x:v>
+      </x:c>
+      <x:c r="B234" t="str">
+        <x:v>听潮</x:v>
+      </x:c>
+      <x:c r="C234" t="str">
+        <x:v>General</x:v>
+      </x:c>
+      <x:c r="D234" t="str">
+        <x:v>ElementTune</x:v>
+      </x:c>
+      <x:c r="E234"/>
+      <x:c r="F234"/>
+      <x:c r="G234" t="str">
+        <x:v>White</x:v>
+      </x:c>
+      <x:c r="H234" t="str">
+        <x:v>Water</x:v>
+      </x:c>
+      <x:c r="I234" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J234" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K234" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L234" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M234" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N234" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O234" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P234" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q234" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R234" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S234" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T234" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U234" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="V234" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W234" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X234" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y234" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Z234" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AA234" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="AB234" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="AC234" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AD234" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AE234"/>
+    </x:row>
+    <x:row r="235">
+      <x:c r="A235" t="str">
+        <x:v>ET-WATER-G</x:v>
+      </x:c>
+      <x:c r="B235" t="str">
+        <x:v>引流</x:v>
+      </x:c>
+      <x:c r="C235" t="str">
+        <x:v>General</x:v>
+      </x:c>
+      <x:c r="D235" t="str">
+        <x:v>ElementTune</x:v>
+      </x:c>
+      <x:c r="E235"/>
+      <x:c r="F235"/>
+      <x:c r="G235" t="str">
+        <x:v>Green</x:v>
+      </x:c>
+      <x:c r="H235" t="str">
+        <x:v>Water</x:v>
+      </x:c>
+      <x:c r="I235" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J235" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K235" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L235" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M235" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N235" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O235" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P235" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q235" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R235" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S235" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T235" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U235" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="V235" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W235" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X235" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y235" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Z235" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AA235" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="AB235" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="AC235" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AD235" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AE235"/>
+    </x:row>
+    <x:row r="236">
+      <x:c r="A236" t="str">
+        <x:v>ET-WATER-B</x:v>
+      </x:c>
+      <x:c r="B236" t="str">
+        <x:v>澄波</x:v>
+      </x:c>
+      <x:c r="C236" t="str">
+        <x:v>General</x:v>
+      </x:c>
+      <x:c r="D236" t="str">
+        <x:v>ElementTune</x:v>
+      </x:c>
+      <x:c r="E236"/>
+      <x:c r="F236"/>
+      <x:c r="G236" t="str">
+        <x:v>Blue</x:v>
+      </x:c>
+      <x:c r="H236" t="str">
+        <x:v>Water</x:v>
+      </x:c>
+      <x:c r="I236" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="J236" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K236" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L236" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M236" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="N236" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O236" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P236" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q236" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R236" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S236" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T236" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U236" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="V236" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W236" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X236" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y236" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Z236" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AA236" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AB236" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AC236" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AD236" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AE236"/>
+    </x:row>
+    <x:row r="237">
+      <x:c r="A237" t="str">
+        <x:v>ET-WATER-P</x:v>
+      </x:c>
+      <x:c r="B237" t="str">
+        <x:v>沧海同调</x:v>
+      </x:c>
+      <x:c r="C237" t="str">
+        <x:v>General</x:v>
+      </x:c>
+      <x:c r="D237" t="str">
+        <x:v>ElementTune</x:v>
+      </x:c>
+      <x:c r="E237"/>
+      <x:c r="F237"/>
+      <x:c r="G237" t="str">
+        <x:v>Purple</x:v>
+      </x:c>
+      <x:c r="H237" t="str">
+        <x:v>Water</x:v>
+      </x:c>
+      <x:c r="I237" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="J237" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K237" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L237" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M237" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="N237" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O237" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P237" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q237" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R237" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S237" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T237" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U237" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="V237" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W237" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X237" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y237" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Z237" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AA237" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="AB237" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="AC237" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AD237" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AE237"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -49135,6 +50913,2766 @@
         <x:v>600</x:v>
       </x:c>
       <x:c r="G1205" s="80" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1206">
+      <x:c r="A1206" t="str">
+        <x:v>ET-FIRE-W:0</x:v>
+      </x:c>
+      <x:c r="B1206" t="str">
+        <x:v>ET-FIRE-W</x:v>
+      </x:c>
+      <x:c r="C1206" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D1206" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E1206" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1206" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G1206" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1207">
+      <x:c r="A1207" t="str">
+        <x:v>ET-FIRE-W:1</x:v>
+      </x:c>
+      <x:c r="B1207" t="str">
+        <x:v>ET-FIRE-W</x:v>
+      </x:c>
+      <x:c r="C1207" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D1207" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E1207" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1207" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G1207" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1208">
+      <x:c r="A1208" t="str">
+        <x:v>ET-FIRE-W:2</x:v>
+      </x:c>
+      <x:c r="B1208" t="str">
+        <x:v>ET-FIRE-W</x:v>
+      </x:c>
+      <x:c r="C1208" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D1208" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E1208" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1208" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G1208" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1209">
+      <x:c r="A1209" t="str">
+        <x:v>ET-FIRE-W:3</x:v>
+      </x:c>
+      <x:c r="B1209" t="str">
+        <x:v>ET-FIRE-W</x:v>
+      </x:c>
+      <x:c r="C1209" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D1209" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E1209" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1209" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G1209" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1210">
+      <x:c r="A1210" t="str">
+        <x:v>ET-FIRE-W:4</x:v>
+      </x:c>
+      <x:c r="B1210" t="str">
+        <x:v>ET-FIRE-W</x:v>
+      </x:c>
+      <x:c r="C1210" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D1210" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E1210" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1210" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="G1210" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1211">
+      <x:c r="A1211" t="str">
+        <x:v>ET-FIRE-W:5</x:v>
+      </x:c>
+      <x:c r="B1211" t="str">
+        <x:v>ET-FIRE-W</x:v>
+      </x:c>
+      <x:c r="C1211" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D1211" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E1211" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1211" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="G1211" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1212">
+      <x:c r="A1212" t="str">
+        <x:v>ET-FIRE-G:0</x:v>
+      </x:c>
+      <x:c r="B1212" t="str">
+        <x:v>ET-FIRE-G</x:v>
+      </x:c>
+      <x:c r="C1212" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D1212" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E1212" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1212" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G1212" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1213">
+      <x:c r="A1213" t="str">
+        <x:v>ET-FIRE-G:1</x:v>
+      </x:c>
+      <x:c r="B1213" t="str">
+        <x:v>ET-FIRE-G</x:v>
+      </x:c>
+      <x:c r="C1213" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D1213" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E1213" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1213" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G1213" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1214">
+      <x:c r="A1214" t="str">
+        <x:v>ET-FIRE-G:2</x:v>
+      </x:c>
+      <x:c r="B1214" t="str">
+        <x:v>ET-FIRE-G</x:v>
+      </x:c>
+      <x:c r="C1214" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D1214" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E1214" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1214" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G1214" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1215">
+      <x:c r="A1215" t="str">
+        <x:v>ET-FIRE-G:3</x:v>
+      </x:c>
+      <x:c r="B1215" t="str">
+        <x:v>ET-FIRE-G</x:v>
+      </x:c>
+      <x:c r="C1215" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D1215" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E1215" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1215" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="G1215" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1216">
+      <x:c r="A1216" t="str">
+        <x:v>ET-FIRE-G:4</x:v>
+      </x:c>
+      <x:c r="B1216" t="str">
+        <x:v>ET-FIRE-G</x:v>
+      </x:c>
+      <x:c r="C1216" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D1216" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E1216" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1216" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G1216" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1217">
+      <x:c r="A1217" t="str">
+        <x:v>ET-FIRE-G:5</x:v>
+      </x:c>
+      <x:c r="B1217" t="str">
+        <x:v>ET-FIRE-G</x:v>
+      </x:c>
+      <x:c r="C1217" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D1217" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E1217" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1217" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="G1217" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1218">
+      <x:c r="A1218" t="str">
+        <x:v>ET-FIRE-B:0</x:v>
+      </x:c>
+      <x:c r="B1218" t="str">
+        <x:v>ET-FIRE-B</x:v>
+      </x:c>
+      <x:c r="C1218" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D1218" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E1218" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1218" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G1218" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1219">
+      <x:c r="A1219" t="str">
+        <x:v>ET-FIRE-B:1</x:v>
+      </x:c>
+      <x:c r="B1219" t="str">
+        <x:v>ET-FIRE-B</x:v>
+      </x:c>
+      <x:c r="C1219" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D1219" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E1219" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1219" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="G1219" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1220">
+      <x:c r="A1220" t="str">
+        <x:v>ET-FIRE-B:2</x:v>
+      </x:c>
+      <x:c r="B1220" t="str">
+        <x:v>ET-FIRE-B</x:v>
+      </x:c>
+      <x:c r="C1220" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D1220" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E1220" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1220" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="G1220" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1221">
+      <x:c r="A1221" t="str">
+        <x:v>ET-FIRE-B:3</x:v>
+      </x:c>
+      <x:c r="B1221" t="str">
+        <x:v>ET-FIRE-B</x:v>
+      </x:c>
+      <x:c r="C1221" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D1221" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E1221" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1221" t="n">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="G1221" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1222">
+      <x:c r="A1222" t="str">
+        <x:v>ET-FIRE-B:4</x:v>
+      </x:c>
+      <x:c r="B1222" t="str">
+        <x:v>ET-FIRE-B</x:v>
+      </x:c>
+      <x:c r="C1222" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D1222" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E1222" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1222" t="n">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="G1222" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1223">
+      <x:c r="A1223" t="str">
+        <x:v>ET-FIRE-B:5</x:v>
+      </x:c>
+      <x:c r="B1223" t="str">
+        <x:v>ET-FIRE-B</x:v>
+      </x:c>
+      <x:c r="C1223" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D1223" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E1223" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1223" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="G1223" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1224">
+      <x:c r="A1224" t="str">
+        <x:v>ET-FIRE-P:0</x:v>
+      </x:c>
+      <x:c r="B1224" t="str">
+        <x:v>ET-FIRE-P</x:v>
+      </x:c>
+      <x:c r="C1224" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D1224" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E1224" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1224" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G1224" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1225">
+      <x:c r="A1225" t="str">
+        <x:v>ET-FIRE-P:1</x:v>
+      </x:c>
+      <x:c r="B1225" t="str">
+        <x:v>ET-FIRE-P</x:v>
+      </x:c>
+      <x:c r="C1225" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D1225" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E1225" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1225" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G1225" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1226">
+      <x:c r="A1226" t="str">
+        <x:v>ET-FIRE-P:2</x:v>
+      </x:c>
+      <x:c r="B1226" t="str">
+        <x:v>ET-FIRE-P</x:v>
+      </x:c>
+      <x:c r="C1226" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D1226" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E1226" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1226" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="G1226" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1227">
+      <x:c r="A1227" t="str">
+        <x:v>ET-FIRE-P:3</x:v>
+      </x:c>
+      <x:c r="B1227" t="str">
+        <x:v>ET-FIRE-P</x:v>
+      </x:c>
+      <x:c r="C1227" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D1227" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E1227" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1227" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="G1227" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1228">
+      <x:c r="A1228" t="str">
+        <x:v>ET-FIRE-P:4</x:v>
+      </x:c>
+      <x:c r="B1228" t="str">
+        <x:v>ET-FIRE-P</x:v>
+      </x:c>
+      <x:c r="C1228" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D1228" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E1228" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1228" t="n">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="G1228" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1229">
+      <x:c r="A1229" t="str">
+        <x:v>ET-FIRE-P:5</x:v>
+      </x:c>
+      <x:c r="B1229" t="str">
+        <x:v>ET-FIRE-P</x:v>
+      </x:c>
+      <x:c r="C1229" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D1229" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E1229" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1229" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="G1229" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1230">
+      <x:c r="A1230" t="str">
+        <x:v>ET-WOOD-W:0</x:v>
+      </x:c>
+      <x:c r="B1230" t="str">
+        <x:v>ET-WOOD-W</x:v>
+      </x:c>
+      <x:c r="C1230" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D1230" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E1230" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1230" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G1230" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1231">
+      <x:c r="A1231" t="str">
+        <x:v>ET-WOOD-W:1</x:v>
+      </x:c>
+      <x:c r="B1231" t="str">
+        <x:v>ET-WOOD-W</x:v>
+      </x:c>
+      <x:c r="C1231" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D1231" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E1231" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1231" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G1231" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1232">
+      <x:c r="A1232" t="str">
+        <x:v>ET-WOOD-W:2</x:v>
+      </x:c>
+      <x:c r="B1232" t="str">
+        <x:v>ET-WOOD-W</x:v>
+      </x:c>
+      <x:c r="C1232" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D1232" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E1232" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1232" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G1232" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1233">
+      <x:c r="A1233" t="str">
+        <x:v>ET-WOOD-W:3</x:v>
+      </x:c>
+      <x:c r="B1233" t="str">
+        <x:v>ET-WOOD-W</x:v>
+      </x:c>
+      <x:c r="C1233" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D1233" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E1233" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1233" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G1233" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1234">
+      <x:c r="A1234" t="str">
+        <x:v>ET-WOOD-W:4</x:v>
+      </x:c>
+      <x:c r="B1234" t="str">
+        <x:v>ET-WOOD-W</x:v>
+      </x:c>
+      <x:c r="C1234" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D1234" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E1234" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1234" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="G1234" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1235">
+      <x:c r="A1235" t="str">
+        <x:v>ET-WOOD-W:5</x:v>
+      </x:c>
+      <x:c r="B1235" t="str">
+        <x:v>ET-WOOD-W</x:v>
+      </x:c>
+      <x:c r="C1235" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D1235" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E1235" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1235" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="G1235" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1236">
+      <x:c r="A1236" t="str">
+        <x:v>ET-WOOD-G:0</x:v>
+      </x:c>
+      <x:c r="B1236" t="str">
+        <x:v>ET-WOOD-G</x:v>
+      </x:c>
+      <x:c r="C1236" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D1236" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E1236" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1236" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G1236" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1237">
+      <x:c r="A1237" t="str">
+        <x:v>ET-WOOD-G:1</x:v>
+      </x:c>
+      <x:c r="B1237" t="str">
+        <x:v>ET-WOOD-G</x:v>
+      </x:c>
+      <x:c r="C1237" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D1237" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E1237" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1237" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G1237" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1238">
+      <x:c r="A1238" t="str">
+        <x:v>ET-WOOD-G:2</x:v>
+      </x:c>
+      <x:c r="B1238" t="str">
+        <x:v>ET-WOOD-G</x:v>
+      </x:c>
+      <x:c r="C1238" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D1238" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E1238" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1238" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G1238" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1239">
+      <x:c r="A1239" t="str">
+        <x:v>ET-WOOD-G:3</x:v>
+      </x:c>
+      <x:c r="B1239" t="str">
+        <x:v>ET-WOOD-G</x:v>
+      </x:c>
+      <x:c r="C1239" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D1239" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E1239" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1239" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="G1239" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1240">
+      <x:c r="A1240" t="str">
+        <x:v>ET-WOOD-G:4</x:v>
+      </x:c>
+      <x:c r="B1240" t="str">
+        <x:v>ET-WOOD-G</x:v>
+      </x:c>
+      <x:c r="C1240" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D1240" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E1240" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1240" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G1240" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1241">
+      <x:c r="A1241" t="str">
+        <x:v>ET-WOOD-G:5</x:v>
+      </x:c>
+      <x:c r="B1241" t="str">
+        <x:v>ET-WOOD-G</x:v>
+      </x:c>
+      <x:c r="C1241" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D1241" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E1241" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1241" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="G1241" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1242">
+      <x:c r="A1242" t="str">
+        <x:v>ET-WOOD-B:0</x:v>
+      </x:c>
+      <x:c r="B1242" t="str">
+        <x:v>ET-WOOD-B</x:v>
+      </x:c>
+      <x:c r="C1242" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D1242" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E1242" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1242" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G1242" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1243">
+      <x:c r="A1243" t="str">
+        <x:v>ET-WOOD-B:1</x:v>
+      </x:c>
+      <x:c r="B1243" t="str">
+        <x:v>ET-WOOD-B</x:v>
+      </x:c>
+      <x:c r="C1243" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D1243" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E1243" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1243" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="G1243" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1244">
+      <x:c r="A1244" t="str">
+        <x:v>ET-WOOD-B:2</x:v>
+      </x:c>
+      <x:c r="B1244" t="str">
+        <x:v>ET-WOOD-B</x:v>
+      </x:c>
+      <x:c r="C1244" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D1244" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E1244" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1244" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="G1244" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1245">
+      <x:c r="A1245" t="str">
+        <x:v>ET-WOOD-B:3</x:v>
+      </x:c>
+      <x:c r="B1245" t="str">
+        <x:v>ET-WOOD-B</x:v>
+      </x:c>
+      <x:c r="C1245" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D1245" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E1245" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1245" t="n">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="G1245" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1246">
+      <x:c r="A1246" t="str">
+        <x:v>ET-WOOD-B:4</x:v>
+      </x:c>
+      <x:c r="B1246" t="str">
+        <x:v>ET-WOOD-B</x:v>
+      </x:c>
+      <x:c r="C1246" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D1246" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E1246" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1246" t="n">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="G1246" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1247">
+      <x:c r="A1247" t="str">
+        <x:v>ET-WOOD-B:5</x:v>
+      </x:c>
+      <x:c r="B1247" t="str">
+        <x:v>ET-WOOD-B</x:v>
+      </x:c>
+      <x:c r="C1247" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D1247" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E1247" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1247" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="G1247" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1248">
+      <x:c r="A1248" t="str">
+        <x:v>ET-WOOD-P:0</x:v>
+      </x:c>
+      <x:c r="B1248" t="str">
+        <x:v>ET-WOOD-P</x:v>
+      </x:c>
+      <x:c r="C1248" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D1248" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E1248" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1248" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G1248" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1249">
+      <x:c r="A1249" t="str">
+        <x:v>ET-WOOD-P:1</x:v>
+      </x:c>
+      <x:c r="B1249" t="str">
+        <x:v>ET-WOOD-P</x:v>
+      </x:c>
+      <x:c r="C1249" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D1249" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E1249" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1249" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G1249" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1250">
+      <x:c r="A1250" t="str">
+        <x:v>ET-WOOD-P:2</x:v>
+      </x:c>
+      <x:c r="B1250" t="str">
+        <x:v>ET-WOOD-P</x:v>
+      </x:c>
+      <x:c r="C1250" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D1250" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E1250" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1250" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="G1250" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1251">
+      <x:c r="A1251" t="str">
+        <x:v>ET-WOOD-P:3</x:v>
+      </x:c>
+      <x:c r="B1251" t="str">
+        <x:v>ET-WOOD-P</x:v>
+      </x:c>
+      <x:c r="C1251" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D1251" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E1251" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1251" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="G1251" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1252">
+      <x:c r="A1252" t="str">
+        <x:v>ET-WOOD-P:4</x:v>
+      </x:c>
+      <x:c r="B1252" t="str">
+        <x:v>ET-WOOD-P</x:v>
+      </x:c>
+      <x:c r="C1252" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D1252" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E1252" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1252" t="n">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="G1252" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1253">
+      <x:c r="A1253" t="str">
+        <x:v>ET-WOOD-P:5</x:v>
+      </x:c>
+      <x:c r="B1253" t="str">
+        <x:v>ET-WOOD-P</x:v>
+      </x:c>
+      <x:c r="C1253" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D1253" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E1253" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1253" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="G1253" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1254">
+      <x:c r="A1254" t="str">
+        <x:v>ET-EARTH-W:0</x:v>
+      </x:c>
+      <x:c r="B1254" t="str">
+        <x:v>ET-EARTH-W</x:v>
+      </x:c>
+      <x:c r="C1254" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D1254" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E1254" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1254" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G1254" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1255">
+      <x:c r="A1255" t="str">
+        <x:v>ET-EARTH-W:1</x:v>
+      </x:c>
+      <x:c r="B1255" t="str">
+        <x:v>ET-EARTH-W</x:v>
+      </x:c>
+      <x:c r="C1255" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D1255" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E1255" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1255" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G1255" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1256">
+      <x:c r="A1256" t="str">
+        <x:v>ET-EARTH-W:2</x:v>
+      </x:c>
+      <x:c r="B1256" t="str">
+        <x:v>ET-EARTH-W</x:v>
+      </x:c>
+      <x:c r="C1256" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D1256" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E1256" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1256" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G1256" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1257">
+      <x:c r="A1257" t="str">
+        <x:v>ET-EARTH-W:3</x:v>
+      </x:c>
+      <x:c r="B1257" t="str">
+        <x:v>ET-EARTH-W</x:v>
+      </x:c>
+      <x:c r="C1257" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D1257" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E1257" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1257" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G1257" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1258">
+      <x:c r="A1258" t="str">
+        <x:v>ET-EARTH-W:4</x:v>
+      </x:c>
+      <x:c r="B1258" t="str">
+        <x:v>ET-EARTH-W</x:v>
+      </x:c>
+      <x:c r="C1258" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D1258" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E1258" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1258" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="G1258" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1259">
+      <x:c r="A1259" t="str">
+        <x:v>ET-EARTH-W:5</x:v>
+      </x:c>
+      <x:c r="B1259" t="str">
+        <x:v>ET-EARTH-W</x:v>
+      </x:c>
+      <x:c r="C1259" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D1259" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E1259" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1259" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="G1259" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1260">
+      <x:c r="A1260" t="str">
+        <x:v>ET-EARTH-G:0</x:v>
+      </x:c>
+      <x:c r="B1260" t="str">
+        <x:v>ET-EARTH-G</x:v>
+      </x:c>
+      <x:c r="C1260" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D1260" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E1260" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1260" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G1260" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1261">
+      <x:c r="A1261" t="str">
+        <x:v>ET-EARTH-G:1</x:v>
+      </x:c>
+      <x:c r="B1261" t="str">
+        <x:v>ET-EARTH-G</x:v>
+      </x:c>
+      <x:c r="C1261" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D1261" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E1261" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1261" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G1261" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1262">
+      <x:c r="A1262" t="str">
+        <x:v>ET-EARTH-G:2</x:v>
+      </x:c>
+      <x:c r="B1262" t="str">
+        <x:v>ET-EARTH-G</x:v>
+      </x:c>
+      <x:c r="C1262" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D1262" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E1262" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1262" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G1262" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1263">
+      <x:c r="A1263" t="str">
+        <x:v>ET-EARTH-G:3</x:v>
+      </x:c>
+      <x:c r="B1263" t="str">
+        <x:v>ET-EARTH-G</x:v>
+      </x:c>
+      <x:c r="C1263" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D1263" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E1263" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1263" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="G1263" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1264">
+      <x:c r="A1264" t="str">
+        <x:v>ET-EARTH-G:4</x:v>
+      </x:c>
+      <x:c r="B1264" t="str">
+        <x:v>ET-EARTH-G</x:v>
+      </x:c>
+      <x:c r="C1264" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D1264" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E1264" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1264" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G1264" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1265">
+      <x:c r="A1265" t="str">
+        <x:v>ET-EARTH-G:5</x:v>
+      </x:c>
+      <x:c r="B1265" t="str">
+        <x:v>ET-EARTH-G</x:v>
+      </x:c>
+      <x:c r="C1265" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D1265" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E1265" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1265" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="G1265" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1266">
+      <x:c r="A1266" t="str">
+        <x:v>ET-EARTH-B:0</x:v>
+      </x:c>
+      <x:c r="B1266" t="str">
+        <x:v>ET-EARTH-B</x:v>
+      </x:c>
+      <x:c r="C1266" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D1266" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E1266" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1266" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G1266" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1267">
+      <x:c r="A1267" t="str">
+        <x:v>ET-EARTH-B:1</x:v>
+      </x:c>
+      <x:c r="B1267" t="str">
+        <x:v>ET-EARTH-B</x:v>
+      </x:c>
+      <x:c r="C1267" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D1267" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E1267" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1267" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="G1267" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1268">
+      <x:c r="A1268" t="str">
+        <x:v>ET-EARTH-B:2</x:v>
+      </x:c>
+      <x:c r="B1268" t="str">
+        <x:v>ET-EARTH-B</x:v>
+      </x:c>
+      <x:c r="C1268" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D1268" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E1268" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1268" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="G1268" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1269">
+      <x:c r="A1269" t="str">
+        <x:v>ET-EARTH-B:3</x:v>
+      </x:c>
+      <x:c r="B1269" t="str">
+        <x:v>ET-EARTH-B</x:v>
+      </x:c>
+      <x:c r="C1269" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D1269" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E1269" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1269" t="n">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="G1269" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1270">
+      <x:c r="A1270" t="str">
+        <x:v>ET-EARTH-B:4</x:v>
+      </x:c>
+      <x:c r="B1270" t="str">
+        <x:v>ET-EARTH-B</x:v>
+      </x:c>
+      <x:c r="C1270" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D1270" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E1270" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1270" t="n">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="G1270" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1271">
+      <x:c r="A1271" t="str">
+        <x:v>ET-EARTH-B:5</x:v>
+      </x:c>
+      <x:c r="B1271" t="str">
+        <x:v>ET-EARTH-B</x:v>
+      </x:c>
+      <x:c r="C1271" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D1271" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E1271" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1271" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="G1271" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1272">
+      <x:c r="A1272" t="str">
+        <x:v>ET-EARTH-P:0</x:v>
+      </x:c>
+      <x:c r="B1272" t="str">
+        <x:v>ET-EARTH-P</x:v>
+      </x:c>
+      <x:c r="C1272" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D1272" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E1272" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1272" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G1272" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1273">
+      <x:c r="A1273" t="str">
+        <x:v>ET-EARTH-P:1</x:v>
+      </x:c>
+      <x:c r="B1273" t="str">
+        <x:v>ET-EARTH-P</x:v>
+      </x:c>
+      <x:c r="C1273" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D1273" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E1273" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1273" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G1273" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1274">
+      <x:c r="A1274" t="str">
+        <x:v>ET-EARTH-P:2</x:v>
+      </x:c>
+      <x:c r="B1274" t="str">
+        <x:v>ET-EARTH-P</x:v>
+      </x:c>
+      <x:c r="C1274" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D1274" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E1274" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1274" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="G1274" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1275">
+      <x:c r="A1275" t="str">
+        <x:v>ET-EARTH-P:3</x:v>
+      </x:c>
+      <x:c r="B1275" t="str">
+        <x:v>ET-EARTH-P</x:v>
+      </x:c>
+      <x:c r="C1275" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D1275" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E1275" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1275" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="G1275" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1276">
+      <x:c r="A1276" t="str">
+        <x:v>ET-EARTH-P:4</x:v>
+      </x:c>
+      <x:c r="B1276" t="str">
+        <x:v>ET-EARTH-P</x:v>
+      </x:c>
+      <x:c r="C1276" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D1276" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E1276" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1276" t="n">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="G1276" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1277">
+      <x:c r="A1277" t="str">
+        <x:v>ET-EARTH-P:5</x:v>
+      </x:c>
+      <x:c r="B1277" t="str">
+        <x:v>ET-EARTH-P</x:v>
+      </x:c>
+      <x:c r="C1277" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D1277" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E1277" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1277" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="G1277" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1278">
+      <x:c r="A1278" t="str">
+        <x:v>ET-METAL-W:0</x:v>
+      </x:c>
+      <x:c r="B1278" t="str">
+        <x:v>ET-METAL-W</x:v>
+      </x:c>
+      <x:c r="C1278" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D1278" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E1278" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1278" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G1278" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1279">
+      <x:c r="A1279" t="str">
+        <x:v>ET-METAL-W:1</x:v>
+      </x:c>
+      <x:c r="B1279" t="str">
+        <x:v>ET-METAL-W</x:v>
+      </x:c>
+      <x:c r="C1279" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D1279" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E1279" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1279" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G1279" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1280">
+      <x:c r="A1280" t="str">
+        <x:v>ET-METAL-W:2</x:v>
+      </x:c>
+      <x:c r="B1280" t="str">
+        <x:v>ET-METAL-W</x:v>
+      </x:c>
+      <x:c r="C1280" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D1280" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E1280" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1280" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G1280" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1281">
+      <x:c r="A1281" t="str">
+        <x:v>ET-METAL-W:3</x:v>
+      </x:c>
+      <x:c r="B1281" t="str">
+        <x:v>ET-METAL-W</x:v>
+      </x:c>
+      <x:c r="C1281" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D1281" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E1281" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1281" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G1281" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1282">
+      <x:c r="A1282" t="str">
+        <x:v>ET-METAL-W:4</x:v>
+      </x:c>
+      <x:c r="B1282" t="str">
+        <x:v>ET-METAL-W</x:v>
+      </x:c>
+      <x:c r="C1282" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D1282" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E1282" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1282" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="G1282" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1283">
+      <x:c r="A1283" t="str">
+        <x:v>ET-METAL-W:5</x:v>
+      </x:c>
+      <x:c r="B1283" t="str">
+        <x:v>ET-METAL-W</x:v>
+      </x:c>
+      <x:c r="C1283" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D1283" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E1283" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1283" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="G1283" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1284">
+      <x:c r="A1284" t="str">
+        <x:v>ET-METAL-G:0</x:v>
+      </x:c>
+      <x:c r="B1284" t="str">
+        <x:v>ET-METAL-G</x:v>
+      </x:c>
+      <x:c r="C1284" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D1284" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E1284" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1284" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G1284" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1285">
+      <x:c r="A1285" t="str">
+        <x:v>ET-METAL-G:1</x:v>
+      </x:c>
+      <x:c r="B1285" t="str">
+        <x:v>ET-METAL-G</x:v>
+      </x:c>
+      <x:c r="C1285" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D1285" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E1285" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1285" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G1285" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1286">
+      <x:c r="A1286" t="str">
+        <x:v>ET-METAL-G:2</x:v>
+      </x:c>
+      <x:c r="B1286" t="str">
+        <x:v>ET-METAL-G</x:v>
+      </x:c>
+      <x:c r="C1286" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D1286" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E1286" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1286" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G1286" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1287">
+      <x:c r="A1287" t="str">
+        <x:v>ET-METAL-G:3</x:v>
+      </x:c>
+      <x:c r="B1287" t="str">
+        <x:v>ET-METAL-G</x:v>
+      </x:c>
+      <x:c r="C1287" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D1287" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E1287" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1287" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="G1287" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1288">
+      <x:c r="A1288" t="str">
+        <x:v>ET-METAL-G:4</x:v>
+      </x:c>
+      <x:c r="B1288" t="str">
+        <x:v>ET-METAL-G</x:v>
+      </x:c>
+      <x:c r="C1288" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D1288" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E1288" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1288" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G1288" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1289">
+      <x:c r="A1289" t="str">
+        <x:v>ET-METAL-G:5</x:v>
+      </x:c>
+      <x:c r="B1289" t="str">
+        <x:v>ET-METAL-G</x:v>
+      </x:c>
+      <x:c r="C1289" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D1289" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E1289" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1289" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="G1289" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1290">
+      <x:c r="A1290" t="str">
+        <x:v>ET-METAL-B:0</x:v>
+      </x:c>
+      <x:c r="B1290" t="str">
+        <x:v>ET-METAL-B</x:v>
+      </x:c>
+      <x:c r="C1290" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D1290" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E1290" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1290" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G1290" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1291">
+      <x:c r="A1291" t="str">
+        <x:v>ET-METAL-B:1</x:v>
+      </x:c>
+      <x:c r="B1291" t="str">
+        <x:v>ET-METAL-B</x:v>
+      </x:c>
+      <x:c r="C1291" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D1291" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E1291" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1291" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="G1291" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1292">
+      <x:c r="A1292" t="str">
+        <x:v>ET-METAL-B:2</x:v>
+      </x:c>
+      <x:c r="B1292" t="str">
+        <x:v>ET-METAL-B</x:v>
+      </x:c>
+      <x:c r="C1292" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D1292" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E1292" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1292" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="G1292" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1293">
+      <x:c r="A1293" t="str">
+        <x:v>ET-METAL-B:3</x:v>
+      </x:c>
+      <x:c r="B1293" t="str">
+        <x:v>ET-METAL-B</x:v>
+      </x:c>
+      <x:c r="C1293" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D1293" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E1293" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1293" t="n">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="G1293" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1294">
+      <x:c r="A1294" t="str">
+        <x:v>ET-METAL-B:4</x:v>
+      </x:c>
+      <x:c r="B1294" t="str">
+        <x:v>ET-METAL-B</x:v>
+      </x:c>
+      <x:c r="C1294" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D1294" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E1294" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1294" t="n">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="G1294" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1295">
+      <x:c r="A1295" t="str">
+        <x:v>ET-METAL-B:5</x:v>
+      </x:c>
+      <x:c r="B1295" t="str">
+        <x:v>ET-METAL-B</x:v>
+      </x:c>
+      <x:c r="C1295" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D1295" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E1295" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1295" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="G1295" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1296">
+      <x:c r="A1296" t="str">
+        <x:v>ET-METAL-P:0</x:v>
+      </x:c>
+      <x:c r="B1296" t="str">
+        <x:v>ET-METAL-P</x:v>
+      </x:c>
+      <x:c r="C1296" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D1296" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E1296" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1296" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G1296" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1297">
+      <x:c r="A1297" t="str">
+        <x:v>ET-METAL-P:1</x:v>
+      </x:c>
+      <x:c r="B1297" t="str">
+        <x:v>ET-METAL-P</x:v>
+      </x:c>
+      <x:c r="C1297" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D1297" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E1297" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1297" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G1297" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1298">
+      <x:c r="A1298" t="str">
+        <x:v>ET-METAL-P:2</x:v>
+      </x:c>
+      <x:c r="B1298" t="str">
+        <x:v>ET-METAL-P</x:v>
+      </x:c>
+      <x:c r="C1298" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D1298" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E1298" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1298" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="G1298" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1299">
+      <x:c r="A1299" t="str">
+        <x:v>ET-METAL-P:3</x:v>
+      </x:c>
+      <x:c r="B1299" t="str">
+        <x:v>ET-METAL-P</x:v>
+      </x:c>
+      <x:c r="C1299" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D1299" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E1299" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1299" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="G1299" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1300">
+      <x:c r="A1300" t="str">
+        <x:v>ET-METAL-P:4</x:v>
+      </x:c>
+      <x:c r="B1300" t="str">
+        <x:v>ET-METAL-P</x:v>
+      </x:c>
+      <x:c r="C1300" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D1300" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E1300" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1300" t="n">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="G1300" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1301">
+      <x:c r="A1301" t="str">
+        <x:v>ET-METAL-P:5</x:v>
+      </x:c>
+      <x:c r="B1301" t="str">
+        <x:v>ET-METAL-P</x:v>
+      </x:c>
+      <x:c r="C1301" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D1301" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E1301" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1301" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="G1301" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1302">
+      <x:c r="A1302" t="str">
+        <x:v>ET-WATER-W:0</x:v>
+      </x:c>
+      <x:c r="B1302" t="str">
+        <x:v>ET-WATER-W</x:v>
+      </x:c>
+      <x:c r="C1302" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D1302" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E1302" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1302" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G1302" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1303">
+      <x:c r="A1303" t="str">
+        <x:v>ET-WATER-W:1</x:v>
+      </x:c>
+      <x:c r="B1303" t="str">
+        <x:v>ET-WATER-W</x:v>
+      </x:c>
+      <x:c r="C1303" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D1303" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E1303" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1303" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G1303" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1304">
+      <x:c r="A1304" t="str">
+        <x:v>ET-WATER-W:2</x:v>
+      </x:c>
+      <x:c r="B1304" t="str">
+        <x:v>ET-WATER-W</x:v>
+      </x:c>
+      <x:c r="C1304" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D1304" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E1304" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1304" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G1304" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1305">
+      <x:c r="A1305" t="str">
+        <x:v>ET-WATER-W:3</x:v>
+      </x:c>
+      <x:c r="B1305" t="str">
+        <x:v>ET-WATER-W</x:v>
+      </x:c>
+      <x:c r="C1305" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D1305" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E1305" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1305" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G1305" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1306">
+      <x:c r="A1306" t="str">
+        <x:v>ET-WATER-W:4</x:v>
+      </x:c>
+      <x:c r="B1306" t="str">
+        <x:v>ET-WATER-W</x:v>
+      </x:c>
+      <x:c r="C1306" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D1306" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E1306" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1306" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="G1306" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1307">
+      <x:c r="A1307" t="str">
+        <x:v>ET-WATER-W:5</x:v>
+      </x:c>
+      <x:c r="B1307" t="str">
+        <x:v>ET-WATER-W</x:v>
+      </x:c>
+      <x:c r="C1307" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D1307" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E1307" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1307" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="G1307" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1308">
+      <x:c r="A1308" t="str">
+        <x:v>ET-WATER-G:0</x:v>
+      </x:c>
+      <x:c r="B1308" t="str">
+        <x:v>ET-WATER-G</x:v>
+      </x:c>
+      <x:c r="C1308" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D1308" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E1308" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1308" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G1308" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1309">
+      <x:c r="A1309" t="str">
+        <x:v>ET-WATER-G:1</x:v>
+      </x:c>
+      <x:c r="B1309" t="str">
+        <x:v>ET-WATER-G</x:v>
+      </x:c>
+      <x:c r="C1309" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D1309" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E1309" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1309" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G1309" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1310">
+      <x:c r="A1310" t="str">
+        <x:v>ET-WATER-G:2</x:v>
+      </x:c>
+      <x:c r="B1310" t="str">
+        <x:v>ET-WATER-G</x:v>
+      </x:c>
+      <x:c r="C1310" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D1310" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E1310" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1310" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G1310" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1311">
+      <x:c r="A1311" t="str">
+        <x:v>ET-WATER-G:3</x:v>
+      </x:c>
+      <x:c r="B1311" t="str">
+        <x:v>ET-WATER-G</x:v>
+      </x:c>
+      <x:c r="C1311" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D1311" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E1311" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1311" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="G1311" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1312">
+      <x:c r="A1312" t="str">
+        <x:v>ET-WATER-G:4</x:v>
+      </x:c>
+      <x:c r="B1312" t="str">
+        <x:v>ET-WATER-G</x:v>
+      </x:c>
+      <x:c r="C1312" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D1312" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E1312" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1312" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G1312" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1313">
+      <x:c r="A1313" t="str">
+        <x:v>ET-WATER-G:5</x:v>
+      </x:c>
+      <x:c r="B1313" t="str">
+        <x:v>ET-WATER-G</x:v>
+      </x:c>
+      <x:c r="C1313" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D1313" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E1313" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1313" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="G1313" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1314">
+      <x:c r="A1314" t="str">
+        <x:v>ET-WATER-B:0</x:v>
+      </x:c>
+      <x:c r="B1314" t="str">
+        <x:v>ET-WATER-B</x:v>
+      </x:c>
+      <x:c r="C1314" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D1314" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E1314" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1314" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G1314" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1315">
+      <x:c r="A1315" t="str">
+        <x:v>ET-WATER-B:1</x:v>
+      </x:c>
+      <x:c r="B1315" t="str">
+        <x:v>ET-WATER-B</x:v>
+      </x:c>
+      <x:c r="C1315" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D1315" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E1315" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1315" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="G1315" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1316">
+      <x:c r="A1316" t="str">
+        <x:v>ET-WATER-B:2</x:v>
+      </x:c>
+      <x:c r="B1316" t="str">
+        <x:v>ET-WATER-B</x:v>
+      </x:c>
+      <x:c r="C1316" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D1316" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E1316" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1316" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="G1316" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1317">
+      <x:c r="A1317" t="str">
+        <x:v>ET-WATER-B:3</x:v>
+      </x:c>
+      <x:c r="B1317" t="str">
+        <x:v>ET-WATER-B</x:v>
+      </x:c>
+      <x:c r="C1317" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D1317" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E1317" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1317" t="n">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="G1317" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1318">
+      <x:c r="A1318" t="str">
+        <x:v>ET-WATER-B:4</x:v>
+      </x:c>
+      <x:c r="B1318" t="str">
+        <x:v>ET-WATER-B</x:v>
+      </x:c>
+      <x:c r="C1318" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D1318" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E1318" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1318" t="n">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="G1318" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1319">
+      <x:c r="A1319" t="str">
+        <x:v>ET-WATER-B:5</x:v>
+      </x:c>
+      <x:c r="B1319" t="str">
+        <x:v>ET-WATER-B</x:v>
+      </x:c>
+      <x:c r="C1319" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D1319" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E1319" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1319" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="G1319" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1320">
+      <x:c r="A1320" t="str">
+        <x:v>ET-WATER-P:0</x:v>
+      </x:c>
+      <x:c r="B1320" t="str">
+        <x:v>ET-WATER-P</x:v>
+      </x:c>
+      <x:c r="C1320" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D1320" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E1320" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1320" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G1320" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1321">
+      <x:c r="A1321" t="str">
+        <x:v>ET-WATER-P:1</x:v>
+      </x:c>
+      <x:c r="B1321" t="str">
+        <x:v>ET-WATER-P</x:v>
+      </x:c>
+      <x:c r="C1321" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D1321" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E1321" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1321" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G1321" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1322">
+      <x:c r="A1322" t="str">
+        <x:v>ET-WATER-P:2</x:v>
+      </x:c>
+      <x:c r="B1322" t="str">
+        <x:v>ET-WATER-P</x:v>
+      </x:c>
+      <x:c r="C1322" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D1322" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E1322" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1322" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="G1322" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1323">
+      <x:c r="A1323" t="str">
+        <x:v>ET-WATER-P:3</x:v>
+      </x:c>
+      <x:c r="B1323" t="str">
+        <x:v>ET-WATER-P</x:v>
+      </x:c>
+      <x:c r="C1323" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D1323" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E1323" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F1323" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="G1323" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1324">
+      <x:c r="A1324" t="str">
+        <x:v>ET-WATER-P:4</x:v>
+      </x:c>
+      <x:c r="B1324" t="str">
+        <x:v>ET-WATER-P</x:v>
+      </x:c>
+      <x:c r="C1324" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D1324" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E1324" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1324" t="n">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="G1324" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1325">
+      <x:c r="A1325" t="str">
+        <x:v>ET-WATER-P:5</x:v>
+      </x:c>
+      <x:c r="B1325" t="str">
+        <x:v>ET-WATER-P</x:v>
+      </x:c>
+      <x:c r="C1325" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D1325" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E1325" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F1325" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="G1325" s="44" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -50447,7 +54985,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a3bedfcedb048d4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c954907027a4e02"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
feat: sync client and server release updates
</commit_message>
<xml_diff>
--- a/config/FantasyCard_Config.xlsx
+++ b/config/FantasyCard_Config.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_README" sheetId="1" r:id="R18397e4dd2f54571"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="2" r:id="R4f4c0111e8c44e5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CardLevels" sheetId="3" r:id="R7edb50c473384c33"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monsters" sheetId="4" r:id="Rcf6deb726ad2481f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterIntents" sheetId="5" r:id="R584031ff52c04ae3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EquipmentQuality" sheetId="6" r:id="R78006436d2a34199"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backpacks" sheetId="7" r:id="Rf35b73f25b5f4d29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LootRules" sheetId="8" r:id="R4e3b41b479424ad4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Economy" sheetId="9" r:id="R0b8ad12cc1e3478c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MapTemplates" sheetId="10" r:id="R52b408d97601403e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BotTuning" sheetId="11" r:id="R47647994d02d4d50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ShopCardPrices" sheetId="12" r:id="Rc4e1fa70431a47dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="13" r:id="R1476ea8a2f244eb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_README" sheetId="1" r:id="Rfd8838a648e84a95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="2" r:id="Rc2d7db1e759745a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CardLevels" sheetId="3" r:id="Re36761b8d2c94f2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monsters" sheetId="4" r:id="R6226a68a12a44a14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterIntents" sheetId="5" r:id="R3f12d0b21a7f4e9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EquipmentQuality" sheetId="6" r:id="R72008fe3c07b4c2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backpacks" sheetId="7" r:id="R89f04c1472f645c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LootRules" sheetId="8" r:id="R5a49124df55d416e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Economy" sheetId="9" r:id="R3bbca8d365f641bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MapTemplates" sheetId="10" r:id="Rda517d91d7c3428e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BotTuning" sheetId="11" r:id="R4642a847146f4150"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ShopCardPrices" sheetId="12" r:id="Rf1ac256b50ff481c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="13" r:id="R508b9c32bf1b4a60"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1476,7 +1476,7 @@
       </x:c>
       <x:c r="C12" s="27" t="n">
         <x:f>COUNTA('Economy'!A6:A205)</x:f>
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -2178,7 +2178,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10e517a74f4d4795"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01350abc2a6c4f73"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -54985,7 +54985,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c954907027a4e02"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b3c3105be654590"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -55802,6 +55802,18 @@
         <x:v>每日 04:00 轮换单卡数量</x:v>
       </x:c>
     </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>daily-shop-refresh-limit</x:v>
+      </x:c>
+      <x:c r="B12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C12"/>
+      <x:c r="D12" t="str">
+        <x:v>商店货架每日可手动刷新次数；按服务器 UTC 0 点重置</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Update game systems and public website
</commit_message>
<xml_diff>
--- a/config/FantasyCard_Config.xlsx
+++ b/config/FantasyCard_Config.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_README" sheetId="1" r:id="Rfd8838a648e84a95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="2" r:id="Rc2d7db1e759745a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CardLevels" sheetId="3" r:id="Re36761b8d2c94f2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monsters" sheetId="4" r:id="R6226a68a12a44a14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterIntents" sheetId="5" r:id="R3f12d0b21a7f4e9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EquipmentQuality" sheetId="6" r:id="R72008fe3c07b4c2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backpacks" sheetId="7" r:id="R89f04c1472f645c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LootRules" sheetId="8" r:id="R5a49124df55d416e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Economy" sheetId="9" r:id="R3bbca8d365f641bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MapTemplates" sheetId="10" r:id="Rda517d91d7c3428e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BotTuning" sheetId="11" r:id="R4642a847146f4150"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ShopCardPrices" sheetId="12" r:id="Rf1ac256b50ff481c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="13" r:id="R508b9c32bf1b4a60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_README" sheetId="1" r:id="R2b0f4400b3c643a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="2" r:id="R4784f469e56e4509"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CardLevels" sheetId="3" r:id="R1804a9364310400f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monsters" sheetId="4" r:id="R636acce276d14e71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterIntents" sheetId="5" r:id="R710d689392044b3e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EquipmentQuality" sheetId="6" r:id="R08438e35c3c74ffc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backpacks" sheetId="7" r:id="R2dd4a51e96714a07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LootRules" sheetId="8" r:id="R765c2417ea2a4482"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Economy" sheetId="9" r:id="R184fa041e5b5469e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MapTemplates" sheetId="10" r:id="Rffece15a73284ba3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BotTuning" sheetId="11" r:id="Rac5a2d32ad074e2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ShopCardPrices" sheetId="12" r:id="R89222dce9df54d8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="13" r:id="Rf19806be86794848"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2178,7 +2178,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01350abc2a6c4f73"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15f24cc493d9494b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -54067,6 +54067,8 @@
     <x:col min="24" max="24" width="18" hidden="0" customWidth="1"/>
     <x:col min="25" max="25" width="18" hidden="0" customWidth="1"/>
     <x:col min="26" max="26" width="18" hidden="0" customWidth="1"/>
+    <x:col min="28" max="28" width="58" hidden="0" customWidth="1"/>
+    <x:col min="29" max="29" width="58" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -54151,6 +54153,12 @@
       <x:c r="AA1" t="str">
         <x:v>display_color</x:v>
       </x:c>
+      <x:c r="AB1" t="str">
+        <x:v>item_background_key</x:v>
+      </x:c>
+      <x:c r="AC1" t="str">
+        <x:v>item_frame_key</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="118" t="str">
@@ -54234,6 +54242,12 @@
       <x:c r="AA2" t="str">
         <x:v>string</x:v>
       </x:c>
+      <x:c r="AB2" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="AC2" t="str">
+        <x:v>string</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="119" t="b">
@@ -54315,6 +54329,12 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="AA3" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AB3" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AC3" s="44" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -54400,6 +54420,12 @@
       <x:c r="AA4" t="str">
         <x:v>client</x:v>
       </x:c>
+      <x:c r="AB4" t="str">
+        <x:v>client</x:v>
+      </x:c>
+      <x:c r="AC4" t="str">
+        <x:v>client</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
       <x:c r="A5" s="124" t="str">
@@ -54483,6 +54509,12 @@
       <x:c r="AA5" t="str">
         <x:v>默认品质色（十六进制）</x:v>
       </x:c>
+      <x:c r="AB5" t="str">
+        <x:v>道具品质底图资源键</x:v>
+      </x:c>
+      <x:c r="AC5" t="str">
+        <x:v>道具品质边框资源键</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="131" t="str">
@@ -54566,6 +54598,12 @@
       <x:c r="AA6" t="str">
         <x:v>#D0C9B6</x:v>
       </x:c>
+      <x:c r="AB6" t="str">
+        <x:v>UI/Prep/exploration_prep_backpack_cell_empty_normal.png</x:v>
+      </x:c>
+      <x:c r="AC6" t="str">
+        <x:v>UI/Prep/exploration_prep_equipment_slot_frame_white.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="131" t="str">
@@ -54649,6 +54687,12 @@
       <x:c r="AA7" t="str">
         <x:v>#789A70</x:v>
       </x:c>
+      <x:c r="AB7" t="str">
+        <x:v>UI/Prep/exploration_prep_backpack_cell_empty_normal.png</x:v>
+      </x:c>
+      <x:c r="AC7" t="str">
+        <x:v>UI/Prep/exploration_prep_equipment_slot_frame_green.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="131" t="str">
@@ -54732,6 +54776,12 @@
       <x:c r="AA8" t="str">
         <x:v>#558CB8</x:v>
       </x:c>
+      <x:c r="AB8" t="str">
+        <x:v>UI/Prep/exploration_prep_backpack_cell_empty_normal.png</x:v>
+      </x:c>
+      <x:c r="AC8" t="str">
+        <x:v>UI/Prep/exploration_prep_equipment_slot_frame_blue.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="131" t="str">
@@ -54815,6 +54865,12 @@
       <x:c r="AA9" t="str">
         <x:v>#9979B1</x:v>
       </x:c>
+      <x:c r="AB9" t="str">
+        <x:v>UI/Prep/exploration_prep_backpack_cell_empty_normal.png</x:v>
+      </x:c>
+      <x:c r="AC9" t="str">
+        <x:v>UI/Prep/exploration_prep_equipment_slot_frame_purple.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="131" t="str">
@@ -54898,6 +54954,12 @@
       <x:c r="AA10" t="str">
         <x:v>#D99B48</x:v>
       </x:c>
+      <x:c r="AB10" t="str">
+        <x:v>UI/Prep/exploration_prep_backpack_cell_empty_normal.png</x:v>
+      </x:c>
+      <x:c r="AC10" t="str">
+        <x:v>UI/Prep/exploration_prep_equipment_slot_frame_orange.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="131" t="str">
@@ -54981,11 +55043,17 @@
       <x:c r="AA11" t="str">
         <x:v>#CE5651</x:v>
       </x:c>
+      <x:c r="AB11" t="str">
+        <x:v>UI/Prep/exploration_prep_backpack_cell_empty_normal.png</x:v>
+      </x:c>
+      <x:c r="AC11" t="str">
+        <x:v>UI/Prep/exploration_prep_equipment_slot_frame_red.png</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b3c3105be654590"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02b34a11de1f48a2"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
feat: integrate bounded monster pool, bot loot, locked policies and client protocol
</commit_message>
<xml_diff>
--- a/config/FantasyCard_Config.xlsx
+++ b/config/FantasyCard_Config.xlsx
@@ -2,19 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_README" sheetId="1" r:id="R2b0f4400b3c643a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="2" r:id="R4784f469e56e4509"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CardLevels" sheetId="3" r:id="R1804a9364310400f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monsters" sheetId="4" r:id="R636acce276d14e71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterIntents" sheetId="5" r:id="R710d689392044b3e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EquipmentQuality" sheetId="6" r:id="R08438e35c3c74ffc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backpacks" sheetId="7" r:id="R2dd4a51e96714a07"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LootRules" sheetId="8" r:id="R765c2417ea2a4482"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Economy" sheetId="9" r:id="R184fa041e5b5469e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MapTemplates" sheetId="10" r:id="Rffece15a73284ba3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BotTuning" sheetId="11" r:id="Rac5a2d32ad074e2e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ShopCardPrices" sheetId="12" r:id="R89222dce9df54d8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="13" r:id="Rf19806be86794848"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_README" sheetId="1" r:id="R4b4b3aa5e90b4bde"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="2" r:id="Ra825414011c64da8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CardLevels" sheetId="3" r:id="R753aadcc67734c53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monsters" sheetId="4" r:id="R935032bdc399417d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterIntents" sheetId="5" r:id="Rf802401b05c64d15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EquipmentQuality" sheetId="6" r:id="Ra22220b041714bd3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backpacks" sheetId="7" r:id="Re2342323c3fe4383"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LootRules" sheetId="8" r:id="R63fc4568409148e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Economy" sheetId="9" r:id="R8d6783d9d769448b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MapTemplates" sheetId="10" r:id="R745c78878207434a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BotTuning" sheetId="11" r:id="R0afbe382f20f46bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ShopCardPrices" sheetId="12" r:id="R2567532650114a7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="13" r:id="Rda4c6f0c9e664a74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NumericalRules" sheetId="14" r:id="R61f905f2113741a2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25,7 +26,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="15">
+  <x:fonts count="16">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -108,8 +109,13 @@
       <x:color rgb="FF1F2937"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="31">
+  <x:fills count="32">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -259,6 +265,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF163B50"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -470,7 +481,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="176">
+  <x:cellXfs count="202">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1031,6 +1042,90 @@
         </x:ext>
       </x:extLst>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -2178,8 +2273,183 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15f24cc493d9494b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re62365f4cb4a4404"/>
   </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="201" t="str">
+        <x:v>id</x:v>
+      </x:c>
+      <x:c r="B1" s="201" t="str">
+        <x:v>cards_spent_draw</x:v>
+      </x:c>
+      <x:c r="C1" s="201" t="str">
+        <x:v>fractional_guardian</x:v>
+      </x:c>
+      <x:c r="D1" s="201" t="str">
+        <x:v>optional_monster_pool</x:v>
+      </x:c>
+      <x:c r="E1" s="201" t="str">
+        <x:v>monster_capacity</x:v>
+      </x:c>
+      <x:c r="F1" s="201" t="str">
+        <x:v>budgeted_bot_loot</x:v>
+      </x:c>
+      <x:c r="G1" s="201" t="str">
+        <x:v>bot_loot_count</x:v>
+      </x:c>
+      <x:c r="H1" s="201" t="str">
+        <x:v>mortal_bot_pve</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="21" customHeight="1">
+      <x:c r="A2" s="174" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="B2" s="174" t="str">
+        <x:v>bool</x:v>
+      </x:c>
+      <x:c r="C2" s="174" t="str">
+        <x:v>bool</x:v>
+      </x:c>
+      <x:c r="D2" s="174" t="str">
+        <x:v>bool</x:v>
+      </x:c>
+      <x:c r="E2" s="174" t="str">
+        <x:v>int64</x:v>
+      </x:c>
+      <x:c r="F2" s="174" t="str">
+        <x:v>bool</x:v>
+      </x:c>
+      <x:c r="G2" s="174" t="str">
+        <x:v>int64</x:v>
+      </x:c>
+      <x:c r="H2" s="174" t="str">
+        <x:v>bool</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="21" customHeight="1">
+      <x:c r="A3" s="175" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B3" s="175" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C3" s="175" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D3" s="175" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E3" s="175" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F3" s="175" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G3" s="175" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H3" s="175" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="21" customHeight="1">
+      <x:c r="A4" s="174" t="str">
+        <x:v>both</x:v>
+      </x:c>
+      <x:c r="B4" s="174" t="str">
+        <x:v>both</x:v>
+      </x:c>
+      <x:c r="C4" s="174" t="str">
+        <x:v>both</x:v>
+      </x:c>
+      <x:c r="D4" s="174" t="str">
+        <x:v>both</x:v>
+      </x:c>
+      <x:c r="E4" s="174" t="str">
+        <x:v>both</x:v>
+      </x:c>
+      <x:c r="F4" s="174" t="str">
+        <x:v>both</x:v>
+      </x:c>
+      <x:c r="G4" s="174" t="str">
+        <x:v>both</x:v>
+      </x:c>
+      <x:c r="H4" s="174" t="str">
+        <x:v>both</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="54" customHeight="1">
+      <x:c r="A5" s="174" t="str">
+        <x:v>生效行；仅一个</x:v>
+      </x:c>
+      <x:c r="B5" s="174" t="str">
+        <x:v>法师按本次实牌返牌；默认关闭</x:v>
+      </x:c>
+      <x:c r="C5" s="174" t="str">
+        <x:v>盾武器余量；默认关闭</x:v>
+      </x:c>
+      <x:c r="D5" s="174" t="str">
+        <x:v>可选怪物卡；默认关闭</x:v>
+      </x:c>
+      <x:c r="E5" s="174" t="str">
+        <x:v>怪物卡上限1—8</x:v>
+      </x:c>
+      <x:c r="F5" s="174" t="str">
+        <x:v>机器人独立战利品；默认关闭</x:v>
+      </x:c>
+      <x:c r="G5" s="174" t="str">
+        <x:v>白绿+0战利品数量0—3</x:v>
+      </x:c>
+      <x:c r="H5" s="174" t="str">
+        <x:v>机器人PVE允许阵亡；默认关闭</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="24" customHeight="1">
+      <x:c r="A6" s="174" t="str">
+        <x:v>current</x:v>
+      </x:c>
+      <x:c r="B6" s="175" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C6" s="175" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D6" s="175" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E6" s="174" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F6" s="175" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G6" s="174" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H6" s="175" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
 
@@ -55053,7 +55323,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02b34a11de1f48a2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5021631cd4a456f"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Revert "Merge remote-tracking branch 'origin/pr/12' into codex/numerical-local-acceptance"
This reverts commit a8815858a63e57aa51e91838674797eef18d146b, reversing
changes made to a234d2e6e76548563aadc10a8da2bd6d9d1c1957.
</commit_message>
<xml_diff>
--- a/config/FantasyCard_Config.xlsx
+++ b/config/FantasyCard_Config.xlsx
@@ -2,20 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_README" sheetId="1" r:id="R4b4b3aa5e90b4bde"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="2" r:id="Ra825414011c64da8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CardLevels" sheetId="3" r:id="R753aadcc67734c53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monsters" sheetId="4" r:id="R935032bdc399417d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterIntents" sheetId="5" r:id="Rf802401b05c64d15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EquipmentQuality" sheetId="6" r:id="Ra22220b041714bd3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backpacks" sheetId="7" r:id="Re2342323c3fe4383"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LootRules" sheetId="8" r:id="R63fc4568409148e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Economy" sheetId="9" r:id="R8d6783d9d769448b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MapTemplates" sheetId="10" r:id="R745c78878207434a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BotTuning" sheetId="11" r:id="R0afbe382f20f46bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ShopCardPrices" sheetId="12" r:id="R2567532650114a7a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="13" r:id="Rda4c6f0c9e664a74"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NumericalRules" sheetId="14" r:id="R61f905f2113741a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_README" sheetId="1" r:id="R2b0f4400b3c643a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="2" r:id="R4784f469e56e4509"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CardLevels" sheetId="3" r:id="R1804a9364310400f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monsters" sheetId="4" r:id="R636acce276d14e71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterIntents" sheetId="5" r:id="R710d689392044b3e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EquipmentQuality" sheetId="6" r:id="R08438e35c3c74ffc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backpacks" sheetId="7" r:id="R2dd4a51e96714a07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LootRules" sheetId="8" r:id="R765c2417ea2a4482"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Economy" sheetId="9" r:id="R184fa041e5b5469e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MapTemplates" sheetId="10" r:id="Rffece15a73284ba3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BotTuning" sheetId="11" r:id="Rac5a2d32ad074e2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ShopCardPrices" sheetId="12" r:id="R89222dce9df54d8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="13" r:id="Rf19806be86794848"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -26,7 +25,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="16">
+  <x:fonts count="15">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -109,13 +108,8 @@
       <x:color rgb="FF1F2937"/>
       <x:name val="Arial"/>
     </x:font>
-    <x:font>
-      <x:sz val="11"/>
-      <x:color rgb="FFFFFFFF"/>
-      <x:name val="Carlito"/>
-    </x:font>
   </x:fonts>
-  <x:fills count="32">
+  <x:fills count="31">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -265,11 +259,6 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF1F4E78"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF163B50"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -481,7 +470,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="202">
+  <x:cellXfs count="176">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1042,90 +1031,6 @@
         </x:ext>
       </x:extLst>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <x:extLst>
-        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
-        </x:ext>
-      </x:extLst>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-      <x:extLst>
-        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
-        </x:ext>
-      </x:extLst>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <x:extLst>
-        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
-        </x:ext>
-      </x:extLst>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-      <x:extLst>
-        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
-        </x:ext>
-      </x:extLst>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <x:extLst>
-        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
-        </x:ext>
-      </x:extLst>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <x:extLst>
-        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
-        </x:ext>
-      </x:extLst>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="10" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="10" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="15" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -2273,183 +2178,8 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re62365f4cb4a4404"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15f24cc493d9494b"/>
   </x:tableParts>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="34" customHeight="1">
-      <x:c r="A1" s="201" t="str">
-        <x:v>id</x:v>
-      </x:c>
-      <x:c r="B1" s="201" t="str">
-        <x:v>cards_spent_draw</x:v>
-      </x:c>
-      <x:c r="C1" s="201" t="str">
-        <x:v>fractional_guardian</x:v>
-      </x:c>
-      <x:c r="D1" s="201" t="str">
-        <x:v>optional_monster_pool</x:v>
-      </x:c>
-      <x:c r="E1" s="201" t="str">
-        <x:v>monster_capacity</x:v>
-      </x:c>
-      <x:c r="F1" s="201" t="str">
-        <x:v>budgeted_bot_loot</x:v>
-      </x:c>
-      <x:c r="G1" s="201" t="str">
-        <x:v>bot_loot_count</x:v>
-      </x:c>
-      <x:c r="H1" s="201" t="str">
-        <x:v>mortal_bot_pve</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="21" customHeight="1">
-      <x:c r="A2" s="174" t="str">
-        <x:v>string</x:v>
-      </x:c>
-      <x:c r="B2" s="174" t="str">
-        <x:v>bool</x:v>
-      </x:c>
-      <x:c r="C2" s="174" t="str">
-        <x:v>bool</x:v>
-      </x:c>
-      <x:c r="D2" s="174" t="str">
-        <x:v>bool</x:v>
-      </x:c>
-      <x:c r="E2" s="174" t="str">
-        <x:v>int64</x:v>
-      </x:c>
-      <x:c r="F2" s="174" t="str">
-        <x:v>bool</x:v>
-      </x:c>
-      <x:c r="G2" s="174" t="str">
-        <x:v>int64</x:v>
-      </x:c>
-      <x:c r="H2" s="174" t="str">
-        <x:v>bool</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="21" customHeight="1">
-      <x:c r="A3" s="175" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B3" s="175" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C3" s="175" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D3" s="175" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E3" s="175" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F3" s="175" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G3" s="175" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H3" s="175" t="b">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="21" customHeight="1">
-      <x:c r="A4" s="174" t="str">
-        <x:v>both</x:v>
-      </x:c>
-      <x:c r="B4" s="174" t="str">
-        <x:v>both</x:v>
-      </x:c>
-      <x:c r="C4" s="174" t="str">
-        <x:v>both</x:v>
-      </x:c>
-      <x:c r="D4" s="174" t="str">
-        <x:v>both</x:v>
-      </x:c>
-      <x:c r="E4" s="174" t="str">
-        <x:v>both</x:v>
-      </x:c>
-      <x:c r="F4" s="174" t="str">
-        <x:v>both</x:v>
-      </x:c>
-      <x:c r="G4" s="174" t="str">
-        <x:v>both</x:v>
-      </x:c>
-      <x:c r="H4" s="174" t="str">
-        <x:v>both</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="54" customHeight="1">
-      <x:c r="A5" s="174" t="str">
-        <x:v>生效行；仅一个</x:v>
-      </x:c>
-      <x:c r="B5" s="174" t="str">
-        <x:v>法师按本次实牌返牌；默认关闭</x:v>
-      </x:c>
-      <x:c r="C5" s="174" t="str">
-        <x:v>盾武器余量；默认关闭</x:v>
-      </x:c>
-      <x:c r="D5" s="174" t="str">
-        <x:v>可选怪物卡；默认关闭</x:v>
-      </x:c>
-      <x:c r="E5" s="174" t="str">
-        <x:v>怪物卡上限1—8</x:v>
-      </x:c>
-      <x:c r="F5" s="174" t="str">
-        <x:v>机器人独立战利品；默认关闭</x:v>
-      </x:c>
-      <x:c r="G5" s="174" t="str">
-        <x:v>白绿+0战利品数量0—3</x:v>
-      </x:c>
-      <x:c r="H5" s="174" t="str">
-        <x:v>机器人PVE允许阵亡；默认关闭</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="24" customHeight="1">
-      <x:c r="A6" s="174" t="str">
-        <x:v>current</x:v>
-      </x:c>
-      <x:c r="B6" s="175" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C6" s="175" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D6" s="175" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E6" s="174" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="F6" s="175" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G6" s="174" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="H6" s="175" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
 
@@ -55323,7 +55053,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5021631cd4a456f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02b34a11de1f48a2"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Reapply "Merge remote-tracking branch 'origin/pr/12' into codex/numerical-local-acceptance"
This reverts commit 97fc677f674b0cd5bb438adbe026c590016cde84.
</commit_message>
<xml_diff>
--- a/config/FantasyCard_Config.xlsx
+++ b/config/FantasyCard_Config.xlsx
@@ -2,19 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_README" sheetId="1" r:id="R2b0f4400b3c643a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="2" r:id="R4784f469e56e4509"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CardLevels" sheetId="3" r:id="R1804a9364310400f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monsters" sheetId="4" r:id="R636acce276d14e71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterIntents" sheetId="5" r:id="R710d689392044b3e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EquipmentQuality" sheetId="6" r:id="R08438e35c3c74ffc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backpacks" sheetId="7" r:id="R2dd4a51e96714a07"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LootRules" sheetId="8" r:id="R765c2417ea2a4482"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Economy" sheetId="9" r:id="R184fa041e5b5469e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MapTemplates" sheetId="10" r:id="Rffece15a73284ba3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BotTuning" sheetId="11" r:id="Rac5a2d32ad074e2e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ShopCardPrices" sheetId="12" r:id="R89222dce9df54d8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="13" r:id="Rf19806be86794848"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_README" sheetId="1" r:id="R4b4b3aa5e90b4bde"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="2" r:id="Ra825414011c64da8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CardLevels" sheetId="3" r:id="R753aadcc67734c53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monsters" sheetId="4" r:id="R935032bdc399417d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterIntents" sheetId="5" r:id="Rf802401b05c64d15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EquipmentQuality" sheetId="6" r:id="Ra22220b041714bd3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backpacks" sheetId="7" r:id="Re2342323c3fe4383"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LootRules" sheetId="8" r:id="R63fc4568409148e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Economy" sheetId="9" r:id="R8d6783d9d769448b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MapTemplates" sheetId="10" r:id="R745c78878207434a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BotTuning" sheetId="11" r:id="R0afbe382f20f46bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ShopCardPrices" sheetId="12" r:id="R2567532650114a7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="13" r:id="Rda4c6f0c9e664a74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NumericalRules" sheetId="14" r:id="R61f905f2113741a2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25,7 +26,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="15">
+  <x:fonts count="16">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -108,8 +109,13 @@
       <x:color rgb="FF1F2937"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="31">
+  <x:fills count="32">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -259,6 +265,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF163B50"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -470,7 +481,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="176">
+  <x:cellXfs count="202">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1031,6 +1042,90 @@
         </x:ext>
       </x:extLst>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -2178,8 +2273,183 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15f24cc493d9494b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re62365f4cb4a4404"/>
   </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="201" t="str">
+        <x:v>id</x:v>
+      </x:c>
+      <x:c r="B1" s="201" t="str">
+        <x:v>cards_spent_draw</x:v>
+      </x:c>
+      <x:c r="C1" s="201" t="str">
+        <x:v>fractional_guardian</x:v>
+      </x:c>
+      <x:c r="D1" s="201" t="str">
+        <x:v>optional_monster_pool</x:v>
+      </x:c>
+      <x:c r="E1" s="201" t="str">
+        <x:v>monster_capacity</x:v>
+      </x:c>
+      <x:c r="F1" s="201" t="str">
+        <x:v>budgeted_bot_loot</x:v>
+      </x:c>
+      <x:c r="G1" s="201" t="str">
+        <x:v>bot_loot_count</x:v>
+      </x:c>
+      <x:c r="H1" s="201" t="str">
+        <x:v>mortal_bot_pve</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="21" customHeight="1">
+      <x:c r="A2" s="174" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="B2" s="174" t="str">
+        <x:v>bool</x:v>
+      </x:c>
+      <x:c r="C2" s="174" t="str">
+        <x:v>bool</x:v>
+      </x:c>
+      <x:c r="D2" s="174" t="str">
+        <x:v>bool</x:v>
+      </x:c>
+      <x:c r="E2" s="174" t="str">
+        <x:v>int64</x:v>
+      </x:c>
+      <x:c r="F2" s="174" t="str">
+        <x:v>bool</x:v>
+      </x:c>
+      <x:c r="G2" s="174" t="str">
+        <x:v>int64</x:v>
+      </x:c>
+      <x:c r="H2" s="174" t="str">
+        <x:v>bool</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="21" customHeight="1">
+      <x:c r="A3" s="175" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B3" s="175" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C3" s="175" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D3" s="175" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E3" s="175" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F3" s="175" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G3" s="175" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H3" s="175" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="21" customHeight="1">
+      <x:c r="A4" s="174" t="str">
+        <x:v>both</x:v>
+      </x:c>
+      <x:c r="B4" s="174" t="str">
+        <x:v>both</x:v>
+      </x:c>
+      <x:c r="C4" s="174" t="str">
+        <x:v>both</x:v>
+      </x:c>
+      <x:c r="D4" s="174" t="str">
+        <x:v>both</x:v>
+      </x:c>
+      <x:c r="E4" s="174" t="str">
+        <x:v>both</x:v>
+      </x:c>
+      <x:c r="F4" s="174" t="str">
+        <x:v>both</x:v>
+      </x:c>
+      <x:c r="G4" s="174" t="str">
+        <x:v>both</x:v>
+      </x:c>
+      <x:c r="H4" s="174" t="str">
+        <x:v>both</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="54" customHeight="1">
+      <x:c r="A5" s="174" t="str">
+        <x:v>生效行；仅一个</x:v>
+      </x:c>
+      <x:c r="B5" s="174" t="str">
+        <x:v>法师按本次实牌返牌；默认关闭</x:v>
+      </x:c>
+      <x:c r="C5" s="174" t="str">
+        <x:v>盾武器余量；默认关闭</x:v>
+      </x:c>
+      <x:c r="D5" s="174" t="str">
+        <x:v>可选怪物卡；默认关闭</x:v>
+      </x:c>
+      <x:c r="E5" s="174" t="str">
+        <x:v>怪物卡上限1—8</x:v>
+      </x:c>
+      <x:c r="F5" s="174" t="str">
+        <x:v>机器人独立战利品；默认关闭</x:v>
+      </x:c>
+      <x:c r="G5" s="174" t="str">
+        <x:v>白绿+0战利品数量0—3</x:v>
+      </x:c>
+      <x:c r="H5" s="174" t="str">
+        <x:v>机器人PVE允许阵亡；默认关闭</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="24" customHeight="1">
+      <x:c r="A6" s="174" t="str">
+        <x:v>current</x:v>
+      </x:c>
+      <x:c r="B6" s="175" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C6" s="175" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D6" s="175" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E6" s="174" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F6" s="175" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G6" s="174" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H6" s="175" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
 
@@ -55053,7 +55323,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02b34a11de1f48a2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5021631cd4a456f"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>